<commit_message>
parchando nuevos items en excel basico productos
</commit_message>
<xml_diff>
--- a/src/data/PRODUCTOS_BASICOS_AUTO.xlsx
+++ b/src/data/PRODUCTOS_BASICOS_AUTO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\WebstormProjects\erpperu2-automation\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D27933BB-7AB9-4134-9C56-88FA2384D6E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51DDD17F-0335-41D2-80F8-B406792F6F38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32025" yWindow="3225" windowWidth="24000" windowHeight="10845" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31590" yWindow="2790" windowWidth="24000" windowHeight="10845" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PRODUCTOS" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="136">
   <si>
     <t>DESCRIPCION</t>
   </si>
@@ -411,6 +411,33 @@
   </si>
   <si>
     <t>STOCK</t>
+  </si>
+  <si>
+    <t>STKPROD001</t>
+  </si>
+  <si>
+    <t>STKPROD002</t>
+  </si>
+  <si>
+    <t>STKPROD003</t>
+  </si>
+  <si>
+    <t>item edicion masivo stock auto</t>
+  </si>
+  <si>
+    <t>imte edicion de stock masivo flexible</t>
+  </si>
+  <si>
+    <t>item para la edicion de stock</t>
+  </si>
+  <si>
+    <t>EDICION</t>
+  </si>
+  <si>
+    <t>MASIVOS</t>
+  </si>
+  <si>
+    <t>AUTO</t>
   </si>
 </sst>
 </file>
@@ -650,7 +677,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -686,6 +713,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1308,46 +1338,118 @@
       </c>
     </row>
     <row r="9" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9"/>
-      <c r="D9"/>
-      <c r="E9"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="15"/>
-      <c r="L9" s="15"/>
+      <c r="A9" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="C9" t="s">
+        <v>133</v>
+      </c>
+      <c r="D9" t="s">
+        <v>134</v>
+      </c>
+      <c r="E9" t="s">
+        <v>135</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J9" s="16">
+        <v>10</v>
+      </c>
+      <c r="K9" s="15">
+        <v>10.5555</v>
+      </c>
+      <c r="L9" s="15">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="10" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10"/>
-      <c r="D10"/>
-      <c r="E10"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="16"/>
-      <c r="K10" s="15"/>
-      <c r="L10" s="15"/>
+      <c r="A10" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D10" t="s">
+        <v>134</v>
+      </c>
+      <c r="E10" t="s">
+        <v>135</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J10" s="16">
+        <v>10</v>
+      </c>
+      <c r="K10" s="15">
+        <v>10.5555</v>
+      </c>
+      <c r="L10" s="15">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="11" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11"/>
-      <c r="D11"/>
-      <c r="E11"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
-      <c r="J11" s="16"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="15"/>
+      <c r="A11" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="C11" t="s">
+        <v>133</v>
+      </c>
+      <c r="D11" t="s">
+        <v>134</v>
+      </c>
+      <c r="E11" t="s">
+        <v>135</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J11" s="16">
+        <v>10</v>
+      </c>
+      <c r="K11" s="15">
+        <v>10.5555</v>
+      </c>
+      <c r="L11" s="15">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="12" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7"/>
@@ -3033,7 +3135,7 @@
           <x14:formula1>
             <xm:f>DOMINIOS!$B$28:$B$43</xm:f>
           </x14:formula1>
-          <xm:sqref>I10:J130</xm:sqref>
+          <xm:sqref>I12:J130</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>